<commit_message>
feat(reto2): add COIL-100 classical ML pipeline, executed notebook, model card PDF and compact 33MB artifact
</commit_message>
<xml_diff>
--- a/docs/deliverables/Entregable_12_Modelo_Costos_FinOps_Azure.xlsx
+++ b/docs/deliverables/Entregable_12_Modelo_Costos_FinOps_Azure.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="1_Parametros_y_Volumetria" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2_Costos_Cloud_Azure_1_Estacion" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3_Escalamiento_1_a_10_Estaciones" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2_Costos_Azure_1_Estacion" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="3_Escalamiento_1_a_10_Est" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="4_Comparativa_Azure_vs_AWS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5_Caso_Negocio_ROI_3_Turnos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
@@ -2115,7 +2115,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="4">
-        <f>'2_Costos_Cloud_Azure_1_Estacion'!F14</f>
+        <f>'2_Costos_Azure_1_Estacion'!F14</f>
         <v/>
       </c>
       <c r="D7" s="4">

</xml_diff>